<commit_message>
feat: trigger-driven evidence policy and refresh G2-16396 artifacts
</commit_message>
<xml_diff>
--- a/uat-test-plans/G2-16396-wishlist-multiple-wl.xlsx
+++ b/uat-test-plans/G2-16396-wishlist-multiple-wl.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>GitHub/commit evidence basis checked via Jira fallback sources (description/comments/issuelinks) for each in-scope story. No explicit PR/commit URLs were found; matrix entries marked Evidence Unavailable.</t>
+          <t>GitHub evidence refresh completed for G2-16396: 13/15 in-scope stories matched to mytheresa/atelier PRs; 2 stories (G2-19106, G2-20842) had no PR hit and remain Evidence Unavailable.</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Multiple in-scope stories provide limited structured AC text, requiring summary-driven validation. No direct PR/commit URLs discovered in retrieved Jira metadata/comments. Wishlist limit behavior is marked configurable/TBC and should be validated exploratorily.</t>
+          <t>G2-19106 and G2-20842: no direct PR match found in mytheresa/atelier by Jira key search. Multiple in-scope stories provide limited structured AC text, requiring summary-driven validation. Wishlist limit behavior is marked configurable/TBC and should be validated exploratorily.</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>payload_bytes=16532; payload_chars=16528; est_tokens~4132; checklist_rows=10; matrix_rows=15; exploratory_rows=3</t>
+          <t>payload_bytes=17758; payload_chars=17754; est_tokens~4439; checklist_rows=10; matrix_rows=15; exploratory_rows=4</t>
         </is>
       </c>
     </row>
@@ -1256,12 +1256,12 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #582 [G2-18231] Wishlist Create/Rename Modal UI (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #702 [G2-18232] Rename WL API Integration (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
@@ -1362,12 +1362,12 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #614 [G2-18233] all wishlist products (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -1415,12 +1415,12 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #629 [G2-18746] Remove wishlist API integration (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -1468,12 +1468,12 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #595 [G2-18799] Create Wish List API integration (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="K6" s="5" t="inlineStr"/>
     </row>
-    <row r="7" ht="34" customHeight="1">
+    <row r="7" ht="49" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>COV-006</t>
@@ -1521,12 +1521,12 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #559 [G2-19105] Add create and edit icons to wishlist nav menu (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>No PR hit found in mytheresa/atelier for Jira key G2-19106; fallback Jira metadata used.</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1631,12 +1631,12 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #569 [G2-19107] Remove wishlist modal (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>No PR hit found in mytheresa/atelier for Jira key G2-20842; fallback Jira metadata used.</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -1741,12 +1741,12 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #596 [G2-21293] Add wishlist selector dropdown on mini PDP (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -1794,12 +1794,12 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #598 [G2-22343] Wishlist navigation improvements (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
@@ -1847,12 +1847,12 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #825 [G2-22969] Delete product from multiple wishlists (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -1900,12 +1900,12 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #845 [G2-23030] Undo product from multiple wishlists (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
@@ -1953,12 +1953,12 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #778 [G2-23523] Default wishlist redirect (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="K15" s="5" t="inlineStr"/>
     </row>
-    <row r="16" ht="34" customHeight="1">
+    <row r="16" ht="49" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>COV-015</t>
@@ -2006,12 +2006,12 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Checked Jira description/comments/issuelinks for PR/commit URLs; none found.</t>
+          <t>PR #776 [G2-23730] Duplicated default wishlist name error text (mytheresa/atelier, closed).</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Evidence Unavailable</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -2032,12 +2032,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
@@ -2093,7 +2093,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="49" customHeight="1">
+    <row r="2" ht="79" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>EXP-001</t>
@@ -2101,27 +2101,27 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Scope Risk</t>
+          <t>Data Integrity</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>G2-16396</t>
+          <t>G2-22969,G2-23030</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Wishlist limits (max lists/items) are noted as configurable/TBC in epic scope text.</t>
+          <t>Delete/Undo behavior across multiple wishlists can regress as list-item relationships change.</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Create additional wishlists and add items until configured cap is approached; observe any threshold message or hard block behavior.</t>
+          <t>Add the same SKU into at least two custom wishlists and All Items. Delete from All Items, verify removal from all linked lists, then trigger Undo immediately and verify restoration in each list.</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>System enforces configured limits gracefully with user-readable messaging and no broken state.</t>
+          <t>Delete removes the SKU from all intended list contexts; Undo restores prior list associations without duplication, stale counters, or ghost entries.</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -2131,16 +2131,16 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>COV-001,COV-005,COV-011</t>
+          <t>COV-012,COV-013</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Epic scope text references configurable list limits and TBC implementation details.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="49" customHeight="1">
+          <t>PR #825 (G2-22969) and PR #845 (G2-23030) in mytheresa/atelier indicate recent high-change surface for relationship consistency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="79" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>EXP-002</t>
@@ -2163,12 +2163,12 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Execute create/rename in MRP acceptance with an error-triggering condition and compare UX against NAP baseline behavior.</t>
+          <t>In MRP acceptance, attempt create/rename with a duplicated list name and with an invalid/edge input. Capture modal error text and recovery path, then compare with NAP behavior for equivalent steps.</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Error copy is actionable and behavior is consistent with brand expectations without trapping the user.</t>
+          <t>MRP shows clear, non-duplicated error text, modal remains recoverable, and user can retry/cancel without losing context.</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Task explicitly calls out MRP-only mismatch scenario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="49" customHeight="1">
+          <t>PR #776 (G2-23730) targets duplicated default wishlist name error text, so wording and recovery should be regression-checked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="64" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>EXP-003</t>
@@ -2210,12 +2210,12 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Start add-to-wishlist while logged out, authenticate, then verify target wishlist selection/action remains coherent post-login.</t>
+          <t>From PDP and MiniPDP while logged out, initiate add-to-wishlist, complete login, and verify post-login continuation preserves the selected target wishlist and pending user intent.</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>No dropped intent, no duplicated actions, and user remains in correct wishlist context.</t>
+          <t>No dropped intent, no duplicate adds, and user lands in a valid wishlist context with expected selector state.</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -2230,7 +2230,54 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Story targets adaptation of prior single-WL auth behavior to multi-WL.</t>
+          <t>No direct PR key hit found for G2-20842 in mytheresa/atelier; keep this as a high-priority exploratory continuity check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="79" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>EXP-004</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Navigation State</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>G2-19105,G2-22343,G2-23523</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Wishlist navigation state can desync across icon actions, truncation/collapse behavior, and single-list redirect.</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Verify create/edit icon visibility by context, long-title truncation and collapse behavior on smaller breakpoints, and direct redirect for single-wishlist accounts from nav entry points.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Navigation controls remain context-correct, long names do not break layout, and single-list users bypass unnecessary selection steps.</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>COV-006,COV-011,COV-014</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>PR #559 (G2-19105), PR #598 (G2-22343), and PR #778 (G2-23523) indicate related navigation behavior areas that should be validated together.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: relax checklist policy and update G2-16396 artifacts
</commit_message>
<xml_diff>
--- a/uat-test-plans/G2-16396-wishlist-multiple-wl.xlsx
+++ b/uat-test-plans/G2-16396-wishlist-multiple-wl.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>20-30 minutes</t>
+          <t>30-45 minutes</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>15 UI-testable child stories mapped to 10 business-journey checklist checks; 16 non-UI/technical or spike stories excluded from business execution scope.</t>
+          <t>15 UI-testable child stories mapped to 16 detailed business checklist checks; 16 non-UI/technical or spike stories excluded from business execution scope.</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>payload_bytes=17758; payload_chars=17754; est_tokens~4439; checklist_rows=10; matrix_rows=15; exploratory_rows=4</t>
+          <t>payload_bytes=20809; payload_chars=20805; est_tokens~5202; checklist_rows=16; matrix_rows=15; exploratory_rows=4</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1133,6 +1133,220 @@
       </c>
       <c r="G11" s="5" t="inlineStr"/>
       <c r="H11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12" ht="64" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>UAT-011</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Aguilar Sayaan, Nicholas || LuxExperience.com</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Default Wishlist Guardrails</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Default wishlist cannot be renamed or removed</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>1. Open the default wishlist and inspect available actions in wishlist navigation/edit controls.
+2. Compare against a custom wishlist.</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Default wishlist does not expose Rename/Remove actions.
+Custom wishlists expose Rename/Remove in expected contexts.</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr"/>
+      <c r="H12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13" ht="64" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>UAT-012</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Aguilar Sayaan, Nicholas || LuxExperience.com</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Modal Validation</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Create/Rename modal validates duplicate name behavior and displays clear error state</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>1. Attempt to create or rename a wishlist using a name that already exists.
+2. Observe inline validation text, field styling, and retry behavior.</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Duplicate name attempt is blocked with clear inline error text.
+User can correct input and submit successfully without refreshing.</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14" ht="64" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>UAT-013</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Aguilar Sayaan, Nicholas || LuxExperience.com</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Modal Cancel Safety</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Cancel or close actions in create/rename/remove modals do not mutate data</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>1. Open create/rename/remove modal flows and dismiss via Cancel and close icon.
+2. Re-open list state and verify no rename, create, or remove was applied.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Dismissing modal performs no mutation.
+List names and membership remain unchanged after cancel/close.</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15" ht="64" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>UAT-014</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Aguilar Sayaan, Nicholas || LuxExperience.com</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Post-Remove Stability</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>After removing a custom wishlist, user lands in a stable fallback view</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>1. Remove a custom wishlist while viewing it.
+2. Verify landing context (remaining list/all-items), selected navigation state, and absence of broken links.</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>User is redirected to a valid remaining context after removal.
+No broken or stale selected-list state remains.</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16" ht="64" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>UAT-015</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Aguilar Sayaan, Nicholas || LuxExperience.com</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>MiniPDP Targeting</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>MiniPDP wishlist dropdown adds product to the explicitly selected list</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>From MiniPDP with multiple wishlists, choose a non-default target list, add item, then navigate to that list and at least one other list.</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Item appears in selected target wishlist.
+Item does not appear in unrelated list unless previously saved there.</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr"/>
+      <c r="H16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17" ht="64" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>UAT-016</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Aguilar Sayaan, Nicholas || LuxExperience.com</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>All Items Consistency</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>All-items counts and membership stay consistent after delete and undo across multiple lists</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Save one product into multiple wishlists, delete it from All Items, confirm counters/membership updates, then undo and verify full restoration.</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Delete updates list membership and counters consistently.
+Undo restores previous membership/counter state without duplicates.</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1153,7 +1367,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
@@ -1246,7 +1460,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>UAT-001,UAT-002</t>
+          <t>UAT-001,UAT-002,UAT-012,UAT-013</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -1299,7 +1513,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>UAT-002</t>
+          <t>UAT-002,UAT-012</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -1352,7 +1566,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>UAT-006</t>
+          <t>UAT-006,UAT-016</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -1405,7 +1619,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>UAT-003</t>
+          <t>UAT-003,UAT-013,UAT-014</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -1511,7 +1725,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>UAT-004</t>
+          <t>UAT-004,UAT-011</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -1621,7 +1835,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>UAT-003</t>
+          <t>UAT-003,UAT-013</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -1731,7 +1945,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>UAT-005</t>
+          <t>UAT-005,UAT-015</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -1837,7 +2051,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>UAT-009</t>
+          <t>UAT-009,UAT-016</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -1890,7 +2104,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>UAT-010</t>
+          <t>UAT-010,UAT-016</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1996,7 +2210,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>UAT-010</t>
+          <t>UAT-010,UAT-012</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">

</xml_diff>